<commit_message>
Added Traditional Test Cases
</commit_message>
<xml_diff>
--- a/TestCases/Gmail_Compose_Test_Cases.xlsx
+++ b/TestCases/Gmail_Compose_Test_Cases.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/A3B9C077B049E798/ドキュメント/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="8_{0286DDE1-E802-41A7-9A2F-96697CFB64E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B16A896-24F4-4606-A0E2-163061641910}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="8_{0286DDE1-E802-41A7-9A2F-96697CFB64E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45B4B408-5749-4F89-A3A0-4A33592A5B7B}"/>
   <bookViews>
-    <workbookView xWindow="-50475" yWindow="-8925" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-50475" yWindow="-8925" windowWidth="38700" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirement Analysis" sheetId="1" r:id="rId1"/>
+    <sheet name="Traditional Test Cases" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="173">
   <si>
     <t>Send Email</t>
   </si>
@@ -134,6 +135,411 @@
   </si>
   <si>
     <t>System should handle network interruption</t>
+  </si>
+  <si>
+    <t>TC ID</t>
+  </si>
+  <si>
+    <t>Test Scenario</t>
+  </si>
+  <si>
+    <t>Test Data</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>TC001</t>
+  </si>
+  <si>
+    <t>Open Compose Window</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Compose window opens successfully</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>TC002</t>
+  </si>
+  <si>
+    <t>Verify Compose window UI elements</t>
+  </si>
+  <si>
+    <t>To, Subject, Body and Send button displayed</t>
+  </si>
+  <si>
+    <t>TC003</t>
+  </si>
+  <si>
+    <t>Enter valid recipient email</t>
+  </si>
+  <si>
+    <t>test@gmail.com</t>
+  </si>
+  <si>
+    <t>Email accepted</t>
+  </si>
+  <si>
+    <t>TC004</t>
+  </si>
+  <si>
+    <t>Enter invalid recipient email</t>
+  </si>
+  <si>
+    <t>abc.com</t>
+  </si>
+  <si>
+    <t>Validation message displayed</t>
+  </si>
+  <si>
+    <t>TC005</t>
+  </si>
+  <si>
+    <t>Enter email without domain</t>
+  </si>
+  <si>
+    <t>test@</t>
+  </si>
+  <si>
+    <t>TC006</t>
+  </si>
+  <si>
+    <t>Enter email with spaces</t>
+  </si>
+  <si>
+    <t>test @gmail.com</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>TC007</t>
+  </si>
+  <si>
+    <t>Enter multiple valid recipients</t>
+  </si>
+  <si>
+    <t>user1@gmail.com,user2@gmail.com</t>
+  </si>
+  <si>
+    <t>All recipients accepted</t>
+  </si>
+  <si>
+    <t>TC008</t>
+  </si>
+  <si>
+    <t>Leave recipient field blank</t>
+  </si>
+  <si>
+    <t>Blank</t>
+  </si>
+  <si>
+    <t>Email cannot be sent</t>
+  </si>
+  <si>
+    <t>TC009</t>
+  </si>
+  <si>
+    <t>Enter subject "Incubyte"</t>
+  </si>
+  <si>
+    <t>Incubyte</t>
+  </si>
+  <si>
+    <t>Subject accepted</t>
+  </si>
+  <si>
+    <t>TC010</t>
+  </si>
+  <si>
+    <t>Leave subject blank</t>
+  </si>
+  <si>
+    <t>Gmail warning displayed before send</t>
+  </si>
+  <si>
+    <t>TC011</t>
+  </si>
+  <si>
+    <t>Enter very long subject</t>
+  </si>
+  <si>
+    <t>500+ chars</t>
+  </si>
+  <si>
+    <t>Subject handled correctly</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>TC012</t>
+  </si>
+  <si>
+    <t>Enter body text</t>
+  </si>
+  <si>
+    <t>QA test for Incubyte</t>
+  </si>
+  <si>
+    <t>Body accepted</t>
+  </si>
+  <si>
+    <t>TC013</t>
+  </si>
+  <si>
+    <t>Leave body empty</t>
+  </si>
+  <si>
+    <t>Email can still be sent</t>
+  </si>
+  <si>
+    <t>TC014</t>
+  </si>
+  <si>
+    <t>Enter special characters in body</t>
+  </si>
+  <si>
+    <t>!@#$%^&amp;*</t>
+  </si>
+  <si>
+    <t>Characters displayed correctly</t>
+  </si>
+  <si>
+    <t>TC015</t>
+  </si>
+  <si>
+    <t>Enter large body content</t>
+  </si>
+  <si>
+    <t>5000+ chars</t>
+  </si>
+  <si>
+    <t>Content accepted without issue</t>
+  </si>
+  <si>
+    <t>TC016</t>
+  </si>
+  <si>
+    <t>Send email with valid data</t>
+  </si>
+  <si>
+    <t>Valid recipient, subject, body</t>
+  </si>
+  <si>
+    <t>Email sent successfully</t>
+  </si>
+  <si>
+    <t>TC017</t>
+  </si>
+  <si>
+    <t>Verify success notification</t>
+  </si>
+  <si>
+    <t>Valid email</t>
+  </si>
+  <si>
+    <t>TC018</t>
+  </si>
+  <si>
+    <t>Click Send multiple times rapidly</t>
+  </si>
+  <si>
+    <t>Valid data</t>
+  </si>
+  <si>
+    <t>Only one email sent</t>
+  </si>
+  <si>
+    <t>TC019</t>
+  </si>
+  <si>
+    <t>Send email with blank recipient</t>
+  </si>
+  <si>
+    <t>Blank recipient</t>
+  </si>
+  <si>
+    <t>Validation displayed</t>
+  </si>
+  <si>
+    <t>TC020</t>
+  </si>
+  <si>
+    <t>Save draft by closing compose window</t>
+  </si>
+  <si>
+    <t>Valid content</t>
+  </si>
+  <si>
+    <t>Draft saved successfully</t>
+  </si>
+  <si>
+    <t>TC021</t>
+  </si>
+  <si>
+    <t>Open saved draft</t>
+  </si>
+  <si>
+    <t>Existing draft</t>
+  </si>
+  <si>
+    <t>Draft content retained</t>
+  </si>
+  <si>
+    <t>TC022</t>
+  </si>
+  <si>
+    <t>Verify auto-save draft functionality</t>
+  </si>
+  <si>
+    <t>Draft auto-saved</t>
+  </si>
+  <si>
+    <t>TC023</t>
+  </si>
+  <si>
+    <t>Refresh browser while composing</t>
+  </si>
+  <si>
+    <t>Draft content entered</t>
+  </si>
+  <si>
+    <t>Draft recoverable</t>
+  </si>
+  <si>
+    <t>TC024</t>
+  </si>
+  <si>
+    <t>Close browser while composing</t>
+  </si>
+  <si>
+    <t>Draft available after reopening Gmail</t>
+  </si>
+  <si>
+    <t>TC025</t>
+  </si>
+  <si>
+    <t>Add recipient using contact suggestion</t>
+  </si>
+  <si>
+    <t>Existing contact</t>
+  </si>
+  <si>
+    <t>Contact selected successfully</t>
+  </si>
+  <si>
+    <t>TC026</t>
+  </si>
+  <si>
+    <t>Add CC recipient</t>
+  </si>
+  <si>
+    <t>Valid CC email</t>
+  </si>
+  <si>
+    <t>CC recipient added</t>
+  </si>
+  <si>
+    <t>TC027</t>
+  </si>
+  <si>
+    <t>Add BCC recipient</t>
+  </si>
+  <si>
+    <t>Valid BCC email</t>
+  </si>
+  <si>
+    <t>BCC recipient added</t>
+  </si>
+  <si>
+    <t>TC028</t>
+  </si>
+  <si>
+    <t>Disconnect internet before sending</t>
+  </si>
+  <si>
+    <t>Error displayed / email not sent</t>
+  </si>
+  <si>
+    <t>TC029</t>
+  </si>
+  <si>
+    <t>Reconnect internet and retry sending</t>
+  </si>
+  <si>
+    <t>TC030</t>
+  </si>
+  <si>
+    <t>Verify validation message format</t>
+  </si>
+  <si>
+    <t>Invalid email</t>
+  </si>
+  <si>
+    <t>Appropriate validation shown</t>
+  </si>
+  <si>
+    <t>TC031</t>
+  </si>
+  <si>
+    <t>Copy-paste content into body</t>
+  </si>
+  <si>
+    <t>Text content</t>
+  </si>
+  <si>
+    <t>Content pasted correctly</t>
+  </si>
+  <si>
+    <t>TC032</t>
+  </si>
+  <si>
+    <t>Use keyboard shortcuts while composing</t>
+  </si>
+  <si>
+    <t>Ctrl+C / Ctrl+V</t>
+  </si>
+  <si>
+    <t>Functionality works correctly</t>
+  </si>
+  <si>
+    <t>TC033</t>
+  </si>
+  <si>
+    <t>Send email using keyboard shortcut</t>
+  </si>
+  <si>
+    <t>Ctrl + Enter</t>
+  </si>
+  <si>
+    <t>TC034</t>
+  </si>
+  <si>
+    <t>Minimize compose window</t>
+  </si>
+  <si>
+    <t>Compose minimized successfully</t>
+  </si>
+  <si>
+    <t>TC035</t>
+  </si>
+  <si>
+    <t>Maximize compose window</t>
+  </si>
+  <si>
+    <t>Compose expanded successfully</t>
+  </si>
+  <si>
+    <t>Message Sent notification displayed</t>
   </si>
 </sst>
 </file>
@@ -182,7 +588,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -194,6 +600,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -209,6 +616,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -692,4 +1103,742 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C99572EF-C487-4B1E-B133-753C3C549367}">
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E7" t="s">
+        <v>58</v>
+      </c>
+      <c r="F7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" t="s">
+        <v>68</v>
+      </c>
+      <c r="E8" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E9" t="s">
+        <v>73</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" t="s">
+        <v>80</v>
+      </c>
+      <c r="F11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D12" t="s">
+        <v>83</v>
+      </c>
+      <c r="E12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F12" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" t="s">
+        <v>88</v>
+      </c>
+      <c r="E13" t="s">
+        <v>89</v>
+      </c>
+      <c r="F13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D14" t="s">
+        <v>72</v>
+      </c>
+      <c r="E14" t="s">
+        <v>92</v>
+      </c>
+      <c r="F14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>93</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>94</v>
+      </c>
+      <c r="D15" t="s">
+        <v>95</v>
+      </c>
+      <c r="E15" t="s">
+        <v>96</v>
+      </c>
+      <c r="F15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>98</v>
+      </c>
+      <c r="D16" t="s">
+        <v>99</v>
+      </c>
+      <c r="E16" t="s">
+        <v>100</v>
+      </c>
+      <c r="F16" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" t="s">
+        <v>102</v>
+      </c>
+      <c r="D17" t="s">
+        <v>103</v>
+      </c>
+      <c r="E17" t="s">
+        <v>104</v>
+      </c>
+      <c r="F17" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>105</v>
+      </c>
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" t="s">
+        <v>106</v>
+      </c>
+      <c r="D18" t="s">
+        <v>107</v>
+      </c>
+      <c r="E18" t="s">
+        <v>172</v>
+      </c>
+      <c r="F18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" t="s">
+        <v>109</v>
+      </c>
+      <c r="D19" t="s">
+        <v>110</v>
+      </c>
+      <c r="E19" t="s">
+        <v>111</v>
+      </c>
+      <c r="F19" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>112</v>
+      </c>
+      <c r="B20" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" t="s">
+        <v>113</v>
+      </c>
+      <c r="D20" t="s">
+        <v>114</v>
+      </c>
+      <c r="E20" t="s">
+        <v>115</v>
+      </c>
+      <c r="F20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>116</v>
+      </c>
+      <c r="B21" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" t="s">
+        <v>117</v>
+      </c>
+      <c r="D21" t="s">
+        <v>118</v>
+      </c>
+      <c r="E21" t="s">
+        <v>119</v>
+      </c>
+      <c r="F21" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B22" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" t="s">
+        <v>121</v>
+      </c>
+      <c r="D22" t="s">
+        <v>122</v>
+      </c>
+      <c r="E22" t="s">
+        <v>123</v>
+      </c>
+      <c r="F22" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>124</v>
+      </c>
+      <c r="B23" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" t="s">
+        <v>125</v>
+      </c>
+      <c r="D23" t="s">
+        <v>118</v>
+      </c>
+      <c r="E23" t="s">
+        <v>126</v>
+      </c>
+      <c r="F23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" t="s">
+        <v>128</v>
+      </c>
+      <c r="D24" t="s">
+        <v>129</v>
+      </c>
+      <c r="E24" t="s">
+        <v>130</v>
+      </c>
+      <c r="F24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>131</v>
+      </c>
+      <c r="B25" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" t="s">
+        <v>132</v>
+      </c>
+      <c r="D25" t="s">
+        <v>129</v>
+      </c>
+      <c r="E25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F25" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>134</v>
+      </c>
+      <c r="B26" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" t="s">
+        <v>135</v>
+      </c>
+      <c r="D26" t="s">
+        <v>136</v>
+      </c>
+      <c r="E26" t="s">
+        <v>137</v>
+      </c>
+      <c r="F26" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>138</v>
+      </c>
+      <c r="B27" t="s">
+        <v>32</v>
+      </c>
+      <c r="C27" t="s">
+        <v>139</v>
+      </c>
+      <c r="D27" t="s">
+        <v>140</v>
+      </c>
+      <c r="E27" t="s">
+        <v>141</v>
+      </c>
+      <c r="F27" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>142</v>
+      </c>
+      <c r="B28" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" t="s">
+        <v>143</v>
+      </c>
+      <c r="D28" t="s">
+        <v>144</v>
+      </c>
+      <c r="E28" t="s">
+        <v>145</v>
+      </c>
+      <c r="F28" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>146</v>
+      </c>
+      <c r="B29" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" t="s">
+        <v>147</v>
+      </c>
+      <c r="D29" t="s">
+        <v>107</v>
+      </c>
+      <c r="E29" t="s">
+        <v>148</v>
+      </c>
+      <c r="F29" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>149</v>
+      </c>
+      <c r="B30" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" t="s">
+        <v>150</v>
+      </c>
+      <c r="D30" t="s">
+        <v>107</v>
+      </c>
+      <c r="E30" t="s">
+        <v>104</v>
+      </c>
+      <c r="F30" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>151</v>
+      </c>
+      <c r="B31" t="s">
+        <v>29</v>
+      </c>
+      <c r="C31" t="s">
+        <v>152</v>
+      </c>
+      <c r="D31" t="s">
+        <v>153</v>
+      </c>
+      <c r="E31" t="s">
+        <v>154</v>
+      </c>
+      <c r="F31" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>155</v>
+      </c>
+      <c r="B32" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" t="s">
+        <v>156</v>
+      </c>
+      <c r="D32" t="s">
+        <v>157</v>
+      </c>
+      <c r="E32" t="s">
+        <v>158</v>
+      </c>
+      <c r="F32" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>159</v>
+      </c>
+      <c r="B33" t="s">
+        <v>17</v>
+      </c>
+      <c r="C33" t="s">
+        <v>160</v>
+      </c>
+      <c r="D33" t="s">
+        <v>161</v>
+      </c>
+      <c r="E33" t="s">
+        <v>162</v>
+      </c>
+      <c r="F33" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>163</v>
+      </c>
+      <c r="B34" t="s">
+        <v>20</v>
+      </c>
+      <c r="C34" t="s">
+        <v>164</v>
+      </c>
+      <c r="D34" t="s">
+        <v>165</v>
+      </c>
+      <c r="E34" t="s">
+        <v>104</v>
+      </c>
+      <c r="F34" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>166</v>
+      </c>
+      <c r="B35" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" t="s">
+        <v>167</v>
+      </c>
+      <c r="D35" t="s">
+        <v>45</v>
+      </c>
+      <c r="E35" t="s">
+        <v>168</v>
+      </c>
+      <c r="F35" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>169</v>
+      </c>
+      <c r="B36" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" t="s">
+        <v>170</v>
+      </c>
+      <c r="D36" t="s">
+        <v>45</v>
+      </c>
+      <c r="E36" t="s">
+        <v>171</v>
+      </c>
+      <c r="F36" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add BDD test cases
</commit_message>
<xml_diff>
--- a/TestCases/Gmail_Compose_Test_Cases.xlsx
+++ b/TestCases/Gmail_Compose_Test_Cases.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/A3B9C077B049E798/ドキュメント/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="8_{0286DDE1-E802-41A7-9A2F-96697CFB64E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F104713-AB7B-4FA8-BA91-C85490332DAD}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="8_{0286DDE1-E802-41A7-9A2F-96697CFB64E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5325D78-59AA-41C1-8BC0-9F9A117BC874}"/>
   <bookViews>
-    <workbookView xWindow="-48495" yWindow="-7920" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-47625" yWindow="-6315" windowWidth="38700" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirement Analysis" sheetId="1" r:id="rId1"/>
     <sheet name="Traditional Test Cases" sheetId="2" r:id="rId2"/>
+    <sheet name="BDD Test Cases" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="211">
   <si>
     <t>Send Email</t>
   </si>
@@ -540,6 +541,173 @@
   </si>
   <si>
     <t>Test Case</t>
+  </si>
+  <si>
+    <t>BDD ID</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>BDD Script</t>
+  </si>
+  <si>
+    <t>BDD001</t>
+  </si>
+  <si>
+    <t>Given the user is logged into Gmail
+When the user clicks the Compose button
+Then the Compose email window should open successfully
+And the To field should be displayed
+And the Subject field should be displayed
+And the Message Body field should be displayed</t>
+  </si>
+  <si>
+    <t>BDD002</t>
+  </si>
+  <si>
+    <t>Enter Valid Recipient Email</t>
+  </si>
+  <si>
+    <t>Given the Compose email window is open
+When the user enters a valid email address in the To field
+Then the email address should be accepted
+And no validation error should be displayed</t>
+  </si>
+  <si>
+    <t>BDD003</t>
+  </si>
+  <si>
+    <t>Invalid Recipient Email Validation</t>
+  </si>
+  <si>
+    <t>Given the Compose email window is open
+When the user enters an invalid email address in the To field
+Then a validation error message should be displayed
+And the email should not be eligible for sending</t>
+  </si>
+  <si>
+    <t>BDD004</t>
+  </si>
+  <si>
+    <t>Enter Subject Successfully</t>
+  </si>
+  <si>
+    <t>Given the Compose email window is open
+When the user enters 'Incubyte' in the Subject field
+Then the subject should be displayed correctly
+And the entered value should be retained</t>
+  </si>
+  <si>
+    <t>BDD005</t>
+  </si>
+  <si>
+    <t>Enter Message Body Successfully</t>
+  </si>
+  <si>
+    <t>Given the Compose email window is open
+When the user enters 'QA test for Incubyte' in the Message Body field
+Then the message content should be displayed correctly
+And the entered content should be retained</t>
+  </si>
+  <si>
+    <t>BDD006</t>
+  </si>
+  <si>
+    <t>Send Email Successfully</t>
+  </si>
+  <si>
+    <t>Given the user is composing an email
+And a valid recipient email address is entered
+And the subject is 'Incubyte'
+And the message body is 'QA test for Incubyte'
+When the user clicks the Send button
+Then the email should be sent successfully
+And a Message Sent notification should be displayed</t>
+  </si>
+  <si>
+    <t>BDD007</t>
+  </si>
+  <si>
+    <t>Send Email Without Recipient</t>
+  </si>
+  <si>
+    <t>Given the user is composing an email
+And the subject is 'Incubyte'
+And the message body is 'QA test for Incubyte'
+When the user clicks the Send button
+Then a validation message should be displayed
+And the email should not be sent</t>
+  </si>
+  <si>
+    <t>BDD008</t>
+  </si>
+  <si>
+    <t>Save Email as Draft</t>
+  </si>
+  <si>
+    <t>Given the user is composing an email
+And recipient, subject and message body are entered
+When the user closes the Compose window without sending the email
+Then the email should be saved as a draft
+And the draft should be available in the Drafts folder</t>
+  </si>
+  <si>
+    <t>BDD009</t>
+  </si>
+  <si>
+    <t>Recover Saved Draft</t>
+  </si>
+  <si>
+    <t>Given a draft email already exists
+When the user opens the Drafts folder
+And selects the saved draft
+Then the draft should open successfully
+And all previously entered information should be retained</t>
+  </si>
+  <si>
+    <t>BDD010</t>
+  </si>
+  <si>
+    <t>Add Multiple Recipients</t>
+  </si>
+  <si>
+    <t>Given the Compose email window is open
+When the user enters multiple valid recipient email addresses
+Then all recipient email addresses should be accepted
+And no validation error should be displayed</t>
+  </si>
+  <si>
+    <t>BDD011</t>
+  </si>
+  <si>
+    <t>Network Failure During Send</t>
+  </si>
+  <si>
+    <t>Given the user is composing an email
+And a valid recipient email address is entered
+And the subject is 'Incubyte'
+And the message body is 'QA test for Incubyte'
+When the internet connection is lost
+And the user clicks the Send button
+Then the email should not be sent
+And an appropriate error message should be displayed</t>
+  </si>
+  <si>
+    <t>BDD012</t>
+  </si>
+  <si>
+    <t>Verify Send Confirmation Notification</t>
+  </si>
+  <si>
+    <t>Given the user is composing an email
+And a valid recipient email address is entered
+And the subject is 'Incubyte'
+And the message body is 'QA test for Incubyte'
+When the user clicks the Send button
+Then the email should be sent successfully
+And a Message Sent confirmation notification should be displayed
+And the email should be available in the Sent folder</t>
   </si>
 </sst>
 </file>
@@ -609,7 +777,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -619,6 +787,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1828,4 +1999,202 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EBE5E81-6125-4253-B3BE-4E2B9ABCA0D5}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="100.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>178</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>182</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>184</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>185</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>187</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>190</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>191</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>194</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>196</v>
+      </c>
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
+        <v>197</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>199</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
+        <v>200</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>202</v>
+      </c>
+      <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" t="s">
+        <v>203</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="120" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>205</v>
+      </c>
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" t="s">
+        <v>206</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="120" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>208</v>
+      </c>
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" t="s">
+        <v>209</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>210</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>